<commit_message>
Changes to test scenario 2. Added RS array savin and loading
</commit_message>
<xml_diff>
--- a/Reports/EnvBobLog.xlsx
+++ b/Reports/EnvBobLog.xlsx
@@ -574,10 +574,10 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>97.24842937034347</v>
+        <v>32.18686796864258</v>
       </c>
       <c r="G2" t="n">
-        <v>94.23812941370366</v>
+        <v>29.17656801200277</v>
       </c>
       <c r="H2" t="n">
         <v>1e-30</v>
@@ -586,28 +586,28 @@
         <v>2815.78946910655</v>
       </c>
       <c r="J2" t="n">
-        <v>96.19610472533579</v>
+        <v>31.13454332363488</v>
       </c>
       <c r="K2" t="n">
         <v>187.5468142180631</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>0.9998303855186813</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>-89.70751609533153</v>
       </c>
       <c r="N2" t="n">
-        <v>66.19610472533577</v>
+        <v>1.134543323634884</v>
       </c>
       <c r="O2" t="n">
         <v>30</v>
       </c>
       <c r="P2" t="n">
-        <v>-91.35070949272732</v>
+        <v>-156.4122708944282</v>
       </c>
       <c r="Q2" t="n">
-        <v>-91.35070949272732</v>
+        <v>-156.4122708944282</v>
       </c>
       <c r="R2" t="n">
         <v>4064.853260246761</v>
@@ -631,7 +631,7 @@
         <v>7.535814018149579</v>
       </c>
       <c r="Y2" t="n">
-        <v>163.9731205251298</v>
+        <v>164.9731205251298</v>
       </c>
       <c r="Z2" t="n">
         <v>1.055284896272219</v>
@@ -656,10 +656,10 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>97.26960680290232</v>
+        <v>32.13272442994204</v>
       </c>
       <c r="G3" t="n">
-        <v>94.2593068462625</v>
+        <v>29.12242447330222</v>
       </c>
       <c r="H3" t="n">
         <v>1e-30</v>
@@ -668,28 +668,28 @@
         <v>2808.932536949855</v>
       </c>
       <c r="J3" t="n">
-        <v>96.19610472533579</v>
+        <v>31.0592223523755</v>
       </c>
       <c r="K3" t="n">
         <v>187.5256367855042</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>0.9998092312782793</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>-89.6893696308077</v>
       </c>
       <c r="N3" t="n">
-        <v>66.19610472533577</v>
+        <v>1.059222352375495</v>
       </c>
       <c r="O3" t="n">
         <v>30</v>
       </c>
       <c r="P3" t="n">
-        <v>-91.32953206016848</v>
+        <v>-156.4664144331288</v>
       </c>
       <c r="Q3" t="n">
-        <v>-91.32953206016848</v>
+        <v>-156.4664144331288</v>
       </c>
       <c r="R3" t="n">
         <v>4070.988386033326</v>
@@ -713,10 +713,10 @@
         <v>7.535825022542807</v>
       </c>
       <c r="Y3" t="n">
-        <v>163.951872253482</v>
+        <v>164.951872253482</v>
       </c>
       <c r="Z3" t="n">
-        <v>1.11916110502662</v>
+        <v>1.119161105026607</v>
       </c>
     </row>
     <row r="4">
@@ -738,10 +738,10 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>97.29083503050288</v>
+        <v>32.07326550682729</v>
       </c>
       <c r="G4" t="n">
-        <v>94.28053507386306</v>
+        <v>29.06296555018748</v>
       </c>
       <c r="H4" t="n">
         <v>1e-30</v>
@@ -750,28 +750,28 @@
         <v>2802.075916028852</v>
       </c>
       <c r="J4" t="n">
-        <v>96.19610472533579</v>
+        <v>30.97853520166019</v>
       </c>
       <c r="K4" t="n">
         <v>187.5044085579037</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>0.9997867767228594</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>-89.67112636331564</v>
       </c>
       <c r="N4" t="n">
-        <v>66.19610472533577</v>
+        <v>0.9785352016601896</v>
       </c>
       <c r="O4" t="n">
         <v>30</v>
       </c>
       <c r="P4" t="n">
-        <v>-91.30830383256792</v>
+        <v>-156.5258733562435</v>
       </c>
       <c r="Q4" t="n">
-        <v>-91.30830383256792</v>
+        <v>-156.5258733562435</v>
       </c>
       <c r="R4" t="n">
         <v>4077.118808914962</v>
@@ -795,7 +795,7 @@
         <v>7.535836038587997</v>
       </c>
       <c r="Y4" t="n">
-        <v>163.9305370533707</v>
+        <v>164.9305370533707</v>
       </c>
       <c r="Z4" t="n">
         <v>1.183197228970331</v>
@@ -820,10 +820,10 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>97.31211426277841</v>
+        <v>32.00830851785484</v>
       </c>
       <c r="G5" t="n">
-        <v>94.3018143061386</v>
+        <v>28.99800856121502</v>
       </c>
       <c r="H5" t="n">
         <v>1e-30</v>
@@ -832,28 +832,28 @@
         <v>2795.219618218265</v>
       </c>
       <c r="J5" t="n">
-        <v>96.19610472533579</v>
+        <v>30.8922989804122</v>
       </c>
       <c r="K5" t="n">
         <v>187.4831293256281</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>0.9997630120876797</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>-89.65278546701178</v>
       </c>
       <c r="N5" t="n">
-        <v>66.19610472533577</v>
+        <v>0.8922989804121995</v>
       </c>
       <c r="O5" t="n">
         <v>30</v>
       </c>
       <c r="P5" t="n">
-        <v>-91.28702460029238</v>
+        <v>-156.5908303452159</v>
       </c>
       <c r="Q5" t="n">
-        <v>-91.28702460029238</v>
+        <v>-156.5908303452159</v>
       </c>
       <c r="R5" t="n">
         <v>4083.244521195483</v>
@@ -877,7 +877,7 @@
         <v>7.535847066248904</v>
       </c>
       <c r="Y5" t="n">
-        <v>163.9091141611784</v>
+        <v>164.9091141611784</v>
       </c>
       <c r="Z5" t="n">
         <v>1.247394412869355</v>
@@ -902,10 +902,10 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>97.33344472090315</v>
+        <v>31.9376552141014</v>
       </c>
       <c r="G6" t="n">
-        <v>94.32314476426333</v>
+        <v>28.92735525746158</v>
       </c>
       <c r="H6" t="n">
         <v>1e-30</v>
@@ -914,28 +914,28 @@
         <v>2788.363652149048</v>
       </c>
       <c r="J6" t="n">
-        <v>96.19610472533579</v>
+        <v>30.80031521853403</v>
       </c>
       <c r="K6" t="n">
         <v>187.4617988675034</v>
       </c>
       <c r="L6" t="n">
-        <v>0</v>
+        <v>0.9997379274823645</v>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
+        <v>-89.63434610152402</v>
       </c>
       <c r="N6" t="n">
-        <v>66.19610472533577</v>
+        <v>0.8003152185340365</v>
       </c>
       <c r="O6" t="n">
         <v>30</v>
       </c>
       <c r="P6" t="n">
-        <v>-91.26569414216766</v>
+        <v>-156.6614836489694</v>
       </c>
       <c r="Q6" t="n">
-        <v>-91.26569414216766</v>
+        <v>-156.6614836489694</v>
       </c>
       <c r="R6" t="n">
         <v>4089.365516921297</v>
@@ -959,10 +959,10 @@
         <v>7.535858105489311</v>
       </c>
       <c r="Y6" t="n">
-        <v>163.8876029772208</v>
+        <v>164.8876029772208</v>
       </c>
       <c r="Z6" t="n">
-        <v>1.311753843689576</v>
+        <v>1.311753843689601</v>
       </c>
     </row>
     <row r="7">
@@ -984,10 +984,10 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>97.35482661695511</v>
+        <v>31.86109041358749</v>
       </c>
       <c r="G7" t="n">
-        <v>94.3445266603153</v>
+        <v>28.85079045694768</v>
       </c>
       <c r="H7" t="n">
         <v>1e-30</v>
@@ -996,28 +996,28 @@
         <v>2781.50802986114</v>
       </c>
       <c r="J7" t="n">
-        <v>96.19610472533579</v>
+        <v>30.70236852196818</v>
       </c>
       <c r="K7" t="n">
         <v>187.4404169714515</v>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>0.9997115129086226</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>-89.61580742140809</v>
       </c>
       <c r="N7" t="n">
-        <v>66.19610472533577</v>
+        <v>0.7023685219681762</v>
       </c>
       <c r="O7" t="n">
         <v>30</v>
       </c>
       <c r="P7" t="n">
-        <v>-91.2443122461157</v>
+        <v>-156.7380484494833</v>
       </c>
       <c r="Q7" t="n">
-        <v>-91.2443122461157</v>
+        <v>-156.7380484494833</v>
       </c>
       <c r="R7" t="n">
         <v>4095.481788411548</v>
@@ -1041,7 +1041,7 @@
         <v>7.535869156272923</v>
       </c>
       <c r="Y7" t="n">
-        <v>163.8660027232646</v>
+        <v>164.8660027232646</v>
       </c>
       <c r="Z7" t="n">
         <v>1.376276688121171</v>
@@ -1066,10 +1066,10 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>97.37626016760281</v>
+        <v>31.77838036939573</v>
       </c>
       <c r="G8" t="n">
-        <v>94.365960210963</v>
+        <v>28.76808041275592</v>
       </c>
       <c r="H8" t="n">
         <v>1e-30</v>
@@ -1078,28 +1078,28 @@
         <v>2774.652762393974</v>
       </c>
       <c r="J8" t="n">
-        <v>96.19610472533579</v>
+        <v>30.5982249271287</v>
       </c>
       <c r="K8" t="n">
         <v>187.4189834208038</v>
       </c>
       <c r="L8" t="n">
-        <v>0</v>
+        <v>0.9996837582455187</v>
       </c>
       <c r="M8" t="n">
-        <v>0</v>
+        <v>-89.59716856961302</v>
       </c>
       <c r="N8" t="n">
-        <v>66.19610472533577</v>
+        <v>0.5982249271286952</v>
       </c>
       <c r="O8" t="n">
         <v>30</v>
       </c>
       <c r="P8" t="n">
-        <v>-91.22287869546797</v>
+        <v>-156.820758493675</v>
       </c>
       <c r="Q8" t="n">
-        <v>-91.22287869546797</v>
+        <v>-156.820758493675</v>
       </c>
       <c r="R8" t="n">
         <v>4101.593328551306</v>
@@ -1123,10 +1123,10 @@
         <v>7.535880218563409</v>
       </c>
       <c r="Y8" t="n">
-        <v>163.844312670568</v>
+        <v>164.844312670568</v>
       </c>
       <c r="Z8" t="n">
-        <v>1.440964134184441</v>
+        <v>1.440964134184429</v>
       </c>
     </row>
     <row r="9">
@@ -1148,10 +1148,10 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>97.39774558737386</v>
+        <v>31.68927098393819</v>
       </c>
       <c r="G9" t="n">
-        <v>94.38744563073405</v>
+        <v>28.67897102729838</v>
       </c>
       <c r="H9" t="n">
         <v>1e-30</v>
@@ -1160,28 +1160,28 @@
         <v>2767.797861948103</v>
       </c>
       <c r="J9" t="n">
-        <v>96.19610472533579</v>
+        <v>30.4876301219001</v>
       </c>
       <c r="K9" t="n">
         <v>187.3974980010327</v>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>0.9996546532558847</v>
       </c>
       <c r="M9" t="n">
-        <v>0</v>
+        <v>-89.57842868012946</v>
       </c>
       <c r="N9" t="n">
-        <v>66.19610472533577</v>
+        <v>0.4876301219001064</v>
       </c>
       <c r="O9" t="n">
         <v>30</v>
       </c>
       <c r="P9" t="n">
-        <v>-91.20139327569692</v>
+        <v>-156.9098678791326</v>
       </c>
       <c r="Q9" t="n">
-        <v>-91.20139327569692</v>
+        <v>-156.9098678791326</v>
       </c>
       <c r="R9" t="n">
         <v>4107.700129693329</v>
@@ -1205,7 +1205,7 @@
         <v>7.535891292324466</v>
       </c>
       <c r="Y9" t="n">
-        <v>163.8225320244808</v>
+        <v>164.8225320244808</v>
       </c>
       <c r="Z9" t="n">
         <v>1.505817370914526</v>
@@ -1230,10 +1230,10 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>97.41928310241255</v>
+        <v>31.59348568897201</v>
       </c>
       <c r="G10" t="n">
-        <v>94.40898314577274</v>
+        <v>28.5831857323322</v>
       </c>
       <c r="H10" t="n">
         <v>1e-30</v>
@@ -1242,28 +1242,28 @@
         <v>2760.943337502153</v>
       </c>
       <c r="J10" t="n">
-        <v>96.19610472533579</v>
+        <v>30.37030731189524</v>
       </c>
       <c r="K10" t="n">
         <v>187.375960485994</v>
       </c>
       <c r="L10" t="n">
-        <v>0</v>
+        <v>0.9996241875635582</v>
       </c>
       <c r="M10" t="n">
-        <v>0</v>
+        <v>-89.55958687265007</v>
       </c>
       <c r="N10" t="n">
-        <v>66.19610472533577</v>
+        <v>0.3703073118952399</v>
       </c>
       <c r="O10" t="n">
         <v>30</v>
       </c>
       <c r="P10" t="n">
-        <v>-91.17985576065823</v>
+        <v>-157.0056531740988</v>
       </c>
       <c r="Q10" t="n">
-        <v>-91.17985576065823</v>
+        <v>-157.0056531740988</v>
       </c>
       <c r="R10" t="n">
         <v>4113.802185896458</v>
@@ -1287,7 +1287,7 @@
         <v>7.535902377519727</v>
       </c>
       <c r="Y10" t="n">
-        <v>163.8006601567133</v>
+        <v>164.8006601567133</v>
       </c>
       <c r="Z10" t="n">
         <v>1.570837630214003</v>
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>97.4408729295702</v>
+        <v>31.49072321436286</v>
       </c>
       <c r="G11" t="n">
-        <v>94.43057297293039</v>
+        <v>28.48042325772305</v>
       </c>
       <c r="H11" t="n">
         <v>1e-30</v>
@@ -1324,28 +1324,28 @@
         <v>2754.089201487097</v>
       </c>
       <c r="J11" t="n">
-        <v>96.19610472533579</v>
+        <v>30.24595501012843</v>
       </c>
       <c r="K11" t="n">
         <v>187.3543706588364</v>
       </c>
       <c r="L11" t="n">
-        <v>0</v>
+        <v>0.9995923506849465</v>
       </c>
       <c r="M11" t="n">
-        <v>0</v>
+        <v>-89.54064226057424</v>
       </c>
       <c r="N11" t="n">
-        <v>66.19610472533577</v>
+        <v>0.2459550101284312</v>
       </c>
       <c r="O11" t="n">
         <v>30</v>
       </c>
       <c r="P11" t="n">
-        <v>-91.15826593350057</v>
+        <v>-157.1084156487079</v>
       </c>
       <c r="Q11" t="n">
-        <v>-91.15826593350057</v>
+        <v>-157.1084156487079</v>
       </c>
       <c r="R11" t="n">
         <v>4119.899489477398</v>
@@ -1369,10 +1369,10 @@
         <v>7.53591347411274</v>
       </c>
       <c r="Y11" t="n">
-        <v>163.778696257454</v>
+        <v>164.778696257454</v>
       </c>
       <c r="Z11" t="n">
-        <v>1.636026123521763</v>
+        <v>1.636026123521776</v>
       </c>
     </row>
     <row r="12">
@@ -1394,10 +1394,10 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>97.4625152870881</v>
+        <v>31.38065485199084</v>
       </c>
       <c r="G12" t="n">
-        <v>94.45221533044828</v>
+        <v>28.37035489535102</v>
       </c>
       <c r="H12" t="n">
         <v>1e-30</v>
@@ -1406,28 +1406,28 @@
         <v>2747.235466369206</v>
       </c>
       <c r="J12" t="n">
-        <v>96.19610472533579</v>
+        <v>30.11424429023853</v>
       </c>
       <c r="K12" t="n">
         <v>187.3327283013185</v>
       </c>
       <c r="L12" t="n">
-        <v>0</v>
+        <v>0.9995591320062571</v>
       </c>
       <c r="M12" t="n">
-        <v>0</v>
+        <v>-89.52159394625795</v>
       </c>
       <c r="N12" t="n">
-        <v>66.19610472533577</v>
+        <v>0.1142442902385287</v>
       </c>
       <c r="O12" t="n">
         <v>30</v>
       </c>
       <c r="P12" t="n">
-        <v>-91.13662357598271</v>
+        <v>-157.2184840110799</v>
       </c>
       <c r="Q12" t="n">
-        <v>-91.13662357598271</v>
+        <v>-157.2184840110799</v>
       </c>
       <c r="R12" t="n">
         <v>4125.992032816553</v>
@@ -1451,7 +1451,7 @@
         <v>7.535924582067136</v>
       </c>
       <c r="Y12" t="n">
-        <v>163.75663950775</v>
+        <v>164.75663950775</v>
       </c>
       <c r="Z12" t="n">
         <v>1.70138407432339</v>
@@ -1476,10 +1476,10 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>97.4842104048922</v>
+        <v>31.26292138114069</v>
       </c>
       <c r="G13" t="n">
-        <v>94.47391044825238</v>
+        <v>28.25262142450088</v>
       </c>
       <c r="H13" t="n">
         <v>1e-30</v>
@@ -1488,28 +1488,28 @@
         <v>2740.382141405968</v>
       </c>
       <c r="J13" t="n">
-        <v>96.19610472533579</v>
+        <v>29.97481570158428</v>
       </c>
       <c r="K13" t="n">
         <v>187.3110331835144</v>
       </c>
       <c r="L13" t="n">
-        <v>0</v>
+        <v>0.9995245207745809</v>
       </c>
       <c r="M13" t="n">
-        <v>0</v>
+        <v>-89.50244101794314</v>
       </c>
       <c r="N13" t="n">
-        <v>66.19610472533577</v>
+        <v>-0.02518429841572235</v>
       </c>
       <c r="O13" t="n">
         <v>30</v>
       </c>
       <c r="P13" t="n">
-        <v>-91.11492845817861</v>
+        <v>-157.3362174819301</v>
       </c>
       <c r="Q13" t="n">
-        <v>-91.11492845817861</v>
+        <v>-157.3362174819301</v>
       </c>
       <c r="R13" t="n">
         <v>4132.079809975929</v>
@@ -1533,10 +1533,10 @@
         <v>7.535935701346451</v>
       </c>
       <c r="Y13" t="n">
-        <v>163.7344892568628</v>
+        <v>164.7344892568628</v>
       </c>
       <c r="Z13" t="n">
-        <v>1.766912749526267</v>
+        <v>1.76691274952628</v>
       </c>
     </row>
     <row r="14">
@@ -1558,10 +1558,10 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>97.50595850360671</v>
+        <v>31.13712962278723</v>
       </c>
       <c r="G14" t="n">
-        <v>94.49565854696689</v>
+        <v>28.12682966614742</v>
       </c>
       <c r="H14" t="n">
         <v>1e-30</v>
@@ -1570,28 +1570,28 @@
         <v>2733.529239295291</v>
       </c>
       <c r="J14" t="n">
-        <v>96.19610472533579</v>
+        <v>29.8272758445163</v>
       </c>
       <c r="K14" t="n">
         <v>187.2892850847998</v>
       </c>
       <c r="L14" t="n">
-        <v>0</v>
+        <v>0.9994885061177748</v>
       </c>
       <c r="M14" t="n">
-        <v>0</v>
+        <v>-89.48318255647936</v>
       </c>
       <c r="N14" t="n">
-        <v>66.19610472533577</v>
+        <v>-0.1727241554837027</v>
       </c>
       <c r="O14" t="n">
         <v>30</v>
       </c>
       <c r="P14" t="n">
-        <v>-91.09318035946407</v>
+        <v>-157.4620092402835</v>
       </c>
       <c r="Q14" t="n">
-        <v>-91.09318035946407</v>
+        <v>-157.4620092402835</v>
       </c>
       <c r="R14" t="n">
         <v>4138.162813305039</v>
@@ -1615,10 +1615,10 @@
         <v>7.535946831914168</v>
       </c>
       <c r="Y14" t="n">
-        <v>163.7122446700199</v>
+        <v>164.7122446700199</v>
       </c>
       <c r="Z14" t="n">
-        <v>1.832613395866888</v>
+        <v>1.832613395866875</v>
       </c>
     </row>
     <row r="15">
@@ -1640,10 +1640,10 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>97.52775980873048</v>
+        <v>31.00284835529074</v>
       </c>
       <c r="G15" t="n">
-        <v>94.51745985209067</v>
+        <v>27.99254839865093</v>
       </c>
       <c r="H15" t="n">
         <v>1e-30</v>
@@ -1652,28 +1652,28 @@
         <v>2726.676771686951</v>
       </c>
       <c r="J15" t="n">
-        <v>96.19610472533579</v>
+        <v>29.67119327189604</v>
       </c>
       <c r="K15" t="n">
         <v>187.2674837796761</v>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>0.9994510770300681</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>-89.46381763035788</v>
       </c>
       <c r="N15" t="n">
-        <v>66.19610472533577</v>
+        <v>-0.3288067281039592</v>
       </c>
       <c r="O15" t="n">
         <v>30</v>
       </c>
       <c r="P15" t="n">
-        <v>-91.0713790543403</v>
+        <v>-157.5962905077801</v>
       </c>
       <c r="Q15" t="n">
-        <v>-91.0713790543403</v>
+        <v>-157.5962905077801</v>
       </c>
       <c r="R15" t="n">
         <v>4144.241035757347</v>
@@ -1697,10 +1697,10 @@
         <v>7.535957973733796</v>
       </c>
       <c r="Y15" t="n">
-        <v>163.6899049626078</v>
+        <v>164.6899049626078</v>
       </c>
       <c r="Z15" t="n">
-        <v>1.8984872830552</v>
+        <v>1.898487283055213</v>
       </c>
     </row>
     <row r="16">
@@ -1722,10 +1722,10 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>97.54961454338027</v>
+        <v>30.85960364338833</v>
       </c>
       <c r="G16" t="n">
-        <v>94.53931458674046</v>
+        <v>27.84930368674851</v>
       </c>
       <c r="H16" t="n">
         <v>1e-30</v>
@@ -1734,28 +1734,28 @@
         <v>2719.824751472531</v>
       </c>
       <c r="J16" t="n">
-        <v>96.19610472533579</v>
+        <v>29.50609382534384</v>
       </c>
       <c r="K16" t="n">
         <v>187.2456290450263</v>
       </c>
       <c r="L16" t="n">
-        <v>0</v>
+        <v>0.999412222376258</v>
       </c>
       <c r="M16" t="n">
-        <v>0</v>
+        <v>-89.44434529775604</v>
       </c>
       <c r="N16" t="n">
-        <v>66.19610472533577</v>
+        <v>-0.493906174656159</v>
       </c>
       <c r="O16" t="n">
         <v>30</v>
       </c>
       <c r="P16" t="n">
-        <v>-91.04952431969053</v>
+        <v>-157.7395352196825</v>
       </c>
       <c r="Q16" t="n">
-        <v>-91.04952431969053</v>
+        <v>-157.7395352196825</v>
       </c>
       <c r="R16" t="n">
         <v>4150.314469700492</v>
@@ -1779,10 +1779,10 @@
         <v>7.535969126768791</v>
       </c>
       <c r="Y16" t="n">
-        <v>163.6674692819926</v>
+        <v>164.6674692819926</v>
       </c>
       <c r="Z16" t="n">
-        <v>1.964535681859003</v>
+        <v>1.964535681859015</v>
       </c>
     </row>
     <row r="17">
@@ -1804,10 +1804,10 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>97.5715229426915</v>
+        <v>30.70687330176955</v>
       </c>
       <c r="G17" t="n">
-        <v>94.56122298605169</v>
+        <v>27.69657334512974</v>
       </c>
       <c r="H17" t="n">
         <v>1e-30</v>
@@ -1816,28 +1816,28 @@
         <v>2712.973188276437</v>
       </c>
       <c r="J17" t="n">
-        <v>96.19610472533579</v>
+        <v>29.33145508441383</v>
       </c>
       <c r="K17" t="n">
         <v>187.223720645715</v>
       </c>
       <c r="L17" t="n">
-        <v>0</v>
+        <v>0.9993719308670929</v>
       </c>
       <c r="M17" t="n">
-        <v>0</v>
+        <v>-89.42476460275672</v>
       </c>
       <c r="N17" t="n">
-        <v>66.19610472533577</v>
+        <v>-0.6685449155861717</v>
       </c>
       <c r="O17" t="n">
         <v>30</v>
       </c>
       <c r="P17" t="n">
-        <v>-91.02761592037929</v>
+        <v>-157.8922655613012</v>
       </c>
       <c r="Q17" t="n">
-        <v>-91.02761592037929</v>
+        <v>-157.8922655613012</v>
       </c>
       <c r="R17" t="n">
         <v>4156.383109219659</v>
@@ -1861,10 +1861,10 @@
         <v>7.535980290982569</v>
       </c>
       <c r="Y17" t="n">
-        <v>163.6449369459386</v>
+        <v>164.6449369459386</v>
       </c>
       <c r="Z17" t="n">
-        <v>2.030759907970641</v>
+        <v>2.030759907970616</v>
       </c>
     </row>
     <row r="18">
@@ -1886,10 +1886,10 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>97.59348523238316</v>
+        <v>30.54408065727787</v>
       </c>
       <c r="G18" t="n">
-        <v>94.58318527574335</v>
+        <v>27.53378070063806</v>
       </c>
       <c r="H18" t="n">
         <v>1e-30</v>
@@ -1898,28 +1898,28 @@
         <v>2706.122095179903</v>
       </c>
       <c r="J18" t="n">
-        <v>96.19610472533579</v>
+        <v>29.14670015023048</v>
       </c>
       <c r="K18" t="n">
         <v>187.2017583560234</v>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>0.9993301910937288</v>
       </c>
       <c r="M18" t="n">
-        <v>0</v>
+        <v>-89.40507458061377</v>
       </c>
       <c r="N18" t="n">
-        <v>66.19610472533577</v>
+        <v>-0.853299849769517</v>
       </c>
       <c r="O18" t="n">
         <v>30</v>
       </c>
       <c r="P18" t="n">
-        <v>-91.00565363068762</v>
+        <v>-158.0550582057929</v>
       </c>
       <c r="Q18" t="n">
-        <v>-91.00565363068762</v>
+        <v>-158.0550582057929</v>
       </c>
       <c r="R18" t="n">
         <v>4162.446946698016</v>
@@ -1943,10 +1943,10 @@
         <v>7.535991466338523</v>
       </c>
       <c r="Y18" t="n">
-        <v>163.6223070849084</v>
+        <v>164.6223070849084</v>
       </c>
       <c r="Z18" t="n">
-        <v>2.097161257011621</v>
+        <v>2.097161257011583</v>
       </c>
     </row>
     <row r="19">
@@ -1968,10 +1968,10 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>97.61550163947105</v>
+        <v>30.37058701374187</v>
       </c>
       <c r="G19" t="n">
-        <v>94.60520168283124</v>
+        <v>27.36028705710206</v>
       </c>
       <c r="H19" t="n">
         <v>1e-30</v>
@@ -1980,28 +1980,28 @@
         <v>2699.271485352876</v>
       </c>
       <c r="J19" t="n">
-        <v>96.19610472533579</v>
+        <v>28.95119009960661</v>
       </c>
       <c r="K19" t="n">
         <v>187.1797419489355</v>
       </c>
       <c r="L19" t="n">
-        <v>0</v>
+        <v>0.9992869915093044</v>
       </c>
       <c r="M19" t="n">
-        <v>0</v>
+        <v>-89.38527425452611</v>
       </c>
       <c r="N19" t="n">
-        <v>66.19610472533577</v>
+        <v>-1.048809900393394</v>
       </c>
       <c r="O19" t="n">
         <v>30</v>
       </c>
       <c r="P19" t="n">
-        <v>-90.98363722359976</v>
+        <v>-158.2285518493289</v>
       </c>
       <c r="Q19" t="n">
-        <v>-90.98363722359976</v>
+        <v>-158.2285518493289</v>
       </c>
       <c r="R19" t="n">
         <v>4168.505974541447</v>
@@ -2025,10 +2025,10 @@
         <v>7.536002652800055</v>
       </c>
       <c r="Y19" t="n">
-        <v>163.5995788196273</v>
+        <v>164.5995788196273</v>
       </c>
       <c r="Z19" t="n">
-        <v>2.163741037189362</v>
+        <v>2.16374103718935</v>
       </c>
     </row>
     <row r="20">
@@ -2050,10 +2050,10 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>97.63757240298672</v>
+        <v>30.18568272886018</v>
       </c>
       <c r="G20" t="n">
-        <v>94.62727244634691</v>
+        <v>27.17538277222037</v>
       </c>
       <c r="H20" t="n">
         <v>1e-30</v>
@@ -2062,28 +2062,28 @@
         <v>2692.421368734845</v>
       </c>
       <c r="J20" t="n">
-        <v>96.19610472533579</v>
+        <v>28.74421505120923</v>
       </c>
       <c r="K20" t="n">
         <v>187.1576711854198</v>
       </c>
       <c r="L20" t="n">
-        <v>0</v>
+        <v>0.9992423204035747</v>
       </c>
       <c r="M20" t="n">
-        <v>0</v>
+        <v>-89.36536263381332</v>
       </c>
       <c r="N20" t="n">
-        <v>66.19610472533577</v>
+        <v>-1.255784948790768</v>
       </c>
       <c r="O20" t="n">
         <v>30</v>
       </c>
       <c r="P20" t="n">
-        <v>-90.96156646008407</v>
+        <v>-158.4134561342106</v>
       </c>
       <c r="Q20" t="n">
-        <v>-90.96156646008407</v>
+        <v>-158.4134561342106</v>
       </c>
       <c r="R20" t="n">
         <v>4174.560186828104</v>
@@ -2107,10 +2107,10 @@
         <v>7.536013850330467</v>
       </c>
       <c r="Y20" t="n">
-        <v>163.5767514431665</v>
+        <v>164.5767514431665</v>
       </c>
       <c r="Z20" t="n">
-        <v>2.230500602020816</v>
+        <v>2.230500602020829</v>
       </c>
     </row>
     <row r="21">
@@ -2132,10 +2132,10 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>97.65969775264597</v>
+        <v>29.9885769074284</v>
       </c>
       <c r="G21" t="n">
-        <v>94.64939779600616</v>
+        <v>26.97827695078858</v>
       </c>
       <c r="H21" t="n">
         <v>1e-30</v>
@@ -2144,28 +2144,28 @@
         <v>2685.571758676042</v>
       </c>
       <c r="J21" t="n">
-        <v>96.19610472533579</v>
+        <v>28.5249838801182</v>
       </c>
       <c r="K21" t="n">
         <v>187.1355458357606</v>
       </c>
       <c r="L21" t="n">
-        <v>0</v>
+        <v>0.9991961659424652</v>
       </c>
       <c r="M21" t="n">
-        <v>0</v>
+        <v>-89.34533871766905</v>
       </c>
       <c r="N21" t="n">
-        <v>66.19610472533577</v>
+        <v>-1.4750161198818</v>
       </c>
       <c r="O21" t="n">
         <v>30</v>
       </c>
       <c r="P21" t="n">
-        <v>-90.93944111042482</v>
+        <v>-158.6105619556424</v>
       </c>
       <c r="Q21" t="n">
-        <v>-90.93944111042482</v>
+        <v>-158.6105619556424</v>
       </c>
       <c r="R21" t="n">
         <v>4180.609575994578</v>
@@ -2189,10 +2189,10 @@
         <v>7.536025058893129</v>
       </c>
       <c r="Y21" t="n">
-        <v>163.5538240585597</v>
+        <v>164.5538240585597</v>
       </c>
       <c r="Z21" t="n">
-        <v>2.297441285608205</v>
+        <v>2.297441285608218</v>
       </c>
     </row>
     <row r="22">
@@ -2214,10 +2214,10 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>97.68187792283635</v>
+        <v>29.7783848018303</v>
       </c>
       <c r="G22" t="n">
-        <v>94.67157796619654</v>
+        <v>26.76808484519049</v>
       </c>
       <c r="H22" t="n">
         <v>1e-30</v>
@@ -2226,28 +2226,28 @@
         <v>2678.72266758524</v>
       </c>
       <c r="J22" t="n">
-        <v>96.19610472533579</v>
+        <v>28.29261160432972</v>
       </c>
       <c r="K22" t="n">
         <v>187.1133656655702</v>
       </c>
       <c r="L22" t="n">
-        <v>0</v>
+        <v>0.9991485161412397</v>
       </c>
       <c r="M22" t="n">
-        <v>0</v>
+        <v>-89.32520149252396</v>
       </c>
       <c r="N22" t="n">
-        <v>66.19610472533577</v>
+        <v>-1.707388395670275</v>
       </c>
       <c r="O22" t="n">
         <v>30</v>
       </c>
       <c r="P22" t="n">
-        <v>-90.91726094023444</v>
+        <v>-158.8207540612405</v>
       </c>
       <c r="Q22" t="n">
-        <v>-90.91726094023444</v>
+        <v>-158.8207540612405</v>
       </c>
       <c r="R22" t="n">
         <v>4186.654134981074</v>
@@ -2271,10 +2271,10 @@
         <v>7.536036278451264</v>
       </c>
       <c r="Y22" t="n">
-        <v>163.5307958202829</v>
+        <v>164.5307958202829</v>
       </c>
       <c r="Z22" t="n">
-        <v>2.364564445292857</v>
+        <v>2.364564445292896</v>
       </c>
     </row>
     <row r="23">
@@ -2296,10 +2296,10 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>97.70411314582753</v>
+        <v>29.55411283394943</v>
       </c>
       <c r="G23" t="n">
-        <v>94.69381318918772</v>
+        <v>26.54381287730961</v>
       </c>
       <c r="H23" t="n">
         <v>1e-30</v>
@@ -2308,28 +2308,28 @@
         <v>2671.87410903505</v>
       </c>
       <c r="J23" t="n">
-        <v>96.19610472533579</v>
+        <v>28.04610441345766</v>
       </c>
       <c r="K23" t="n">
         <v>187.091130442579</v>
       </c>
       <c r="L23" t="n">
-        <v>0</v>
+        <v>0.9990993588730406</v>
       </c>
       <c r="M23" t="n">
-        <v>0</v>
+        <v>-89.3049499325263</v>
       </c>
       <c r="N23" t="n">
-        <v>66.19610472533577</v>
+        <v>-1.953895586542343</v>
       </c>
       <c r="O23" t="n">
         <v>30</v>
       </c>
       <c r="P23" t="n">
-        <v>-90.89502571724324</v>
+        <v>-159.0450260291214</v>
       </c>
       <c r="Q23" t="n">
-        <v>-90.89502571724324</v>
+        <v>-159.0450260291214</v>
       </c>
       <c r="R23" t="n">
         <v>4192.693856232201</v>
@@ -2353,7 +2353,7 @@
         <v>7.536047508968182</v>
       </c>
       <c r="Y23" t="n">
-        <v>163.5076658118871</v>
+        <v>164.5076658118871</v>
       </c>
       <c r="Z23" t="n">
         <v>2.431871441127968</v>
@@ -2378,10 +2378,10 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>97.72640366604637</v>
+        <v>29.3146402853062</v>
       </c>
       <c r="G24" t="n">
-        <v>94.71610370940655</v>
+        <v>26.30434032866638</v>
       </c>
       <c r="H24" t="n">
         <v>1e-30</v>
@@ -2390,28 +2390,28 @@
         <v>2665.026093371957</v>
       </c>
       <c r="J24" t="n">
-        <v>96.19610472533579</v>
+        <v>27.7843413445956</v>
       </c>
       <c r="K24" t="n">
         <v>187.0688399223602</v>
       </c>
       <c r="L24" t="n">
-        <v>0</v>
+        <v>0.9990486818376649</v>
       </c>
       <c r="M24" t="n">
-        <v>0</v>
+        <v>-89.28458299814335</v>
       </c>
       <c r="N24" t="n">
-        <v>66.19610472533577</v>
+        <v>-2.215658655404402</v>
       </c>
       <c r="O24" t="n">
         <v>30</v>
       </c>
       <c r="P24" t="n">
-        <v>-90.87273519702441</v>
+        <v>-159.2844985777646</v>
       </c>
       <c r="Q24" t="n">
-        <v>-90.87273519702441</v>
+        <v>-159.2844985777646</v>
       </c>
       <c r="R24" t="n">
         <v>4198.728733844372</v>
@@ -2435,7 +2435,7 @@
         <v>7.536058750407076</v>
       </c>
       <c r="Y24" t="n">
-        <v>163.4844332917572</v>
+        <v>164.4844332917572</v>
       </c>
       <c r="Z24" t="n">
         <v>2.499363679460075</v>
@@ -2460,10 +2460,10 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>97.74874971837355</v>
+        <v>29.05869735166444</v>
       </c>
       <c r="G25" t="n">
-        <v>94.73844976173373</v>
+        <v>26.04839739502463</v>
       </c>
       <c r="H25" t="n">
         <v>1e-30</v>
@@ -2472,28 +2472,28 @@
         <v>2658.178634404458</v>
       </c>
       <c r="J25" t="n">
-        <v>96.19610472533579</v>
+        <v>27.50605235862668</v>
       </c>
       <c r="K25" t="n">
         <v>187.046493870033</v>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>0.9989964726062094</v>
       </c>
       <c r="M25" t="n">
-        <v>0</v>
+        <v>-89.26409963822117</v>
       </c>
       <c r="N25" t="n">
-        <v>66.19610472533577</v>
+        <v>-2.493947641373323</v>
       </c>
       <c r="O25" t="n">
         <v>30</v>
       </c>
       <c r="P25" t="n">
-        <v>-90.85038914469726</v>
+        <v>-159.5404415114064</v>
       </c>
       <c r="Q25" t="n">
-        <v>-90.85038914469726</v>
+        <v>-159.5404415114064</v>
       </c>
       <c r="R25" t="n">
         <v>4204.758760252277</v>
@@ -2517,7 +2517,7 @@
         <v>7.536070002731167</v>
       </c>
       <c r="Y25" t="n">
-        <v>163.46109732498</v>
+        <v>164.46109732498</v>
       </c>
       <c r="Z25" t="n">
         <v>2.567042547016642</v>
@@ -2542,10 +2542,10 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>97.7711515389599</v>
+        <v>28.78483781347484</v>
       </c>
       <c r="G26" t="n">
-        <v>94.76085158232009</v>
+        <v>25.77453785683503</v>
       </c>
       <c r="H26" t="n">
         <v>1e-30</v>
@@ -2554,28 +2554,28 @@
         <v>2651.331746062029</v>
       </c>
       <c r="J26" t="n">
-        <v>96.19610472533579</v>
+        <v>27.20979099985072</v>
       </c>
       <c r="K26" t="n">
         <v>187.0240920494467</v>
       </c>
       <c r="L26" t="n">
-        <v>0</v>
+        <v>0.9989427185964026</v>
       </c>
       <c r="M26" t="n">
-        <v>0</v>
+        <v>-89.24349878833677</v>
       </c>
       <c r="N26" t="n">
-        <v>66.19610472533577</v>
+        <v>-2.79020900014928</v>
       </c>
       <c r="O26" t="n">
         <v>30</v>
       </c>
       <c r="P26" t="n">
-        <v>-90.82798732411089</v>
+        <v>-159.8143010495959</v>
       </c>
       <c r="Q26" t="n">
-        <v>-90.82798732411089</v>
+        <v>-159.8143010495959</v>
       </c>
       <c r="R26" t="n">
         <v>4210.783927892788</v>
@@ -2599,10 +2599,10 @@
         <v>7.536081265903624</v>
       </c>
       <c r="Y26" t="n">
-        <v>163.4376569660906</v>
+        <v>164.4376569660906</v>
       </c>
       <c r="Z26" t="n">
-        <v>2.634909443945255</v>
+        <v>2.63490944394523</v>
       </c>
     </row>
   </sheetData>

</xml_diff>